<commit_message>
NPB自動更新(1軍): 2026-09-09 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/raw/2026-09-09/highlights_20260909.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/raw/2026-09-09/highlights_20260909.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7回裏に勝ち越しの満塁ホームランを放ち、チームを勝利に導いた。</t>
+          <t>7回裏に勝ち越し満塁ホームランを放ち、試合の流れを決定づけた。</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>上沢 直之</t>
+          <t>栗原 陵矢</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>6回を投げ3失点ながら8奪三振の力投で、試合を支配する好投を見せた。</t>
+          <t>3回裏に逆転2ランホームランを放ち、チームを勝利に導く一打となった。</t>
         </is>
       </c>
     </row>
@@ -504,17 +504,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>栗原 陵矢</t>
+          <t>宮﨑 敏郎</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ソフトバンク</t>
+          <t>DeNA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3回裏に逆転の2ランホームランを放ち、試合の流れを大きく引き寄せた。</t>
+          <t>同点ホームランと勝ち越し犠牲フライで、チームの攻撃を牽引した。</t>
         </is>
       </c>
     </row>
@@ -529,17 +529,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>井上 朋也</t>
+          <t>床田 寛樹</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DeNA</t>
+          <t>広島</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6回裏に勝ち越しの3ランホームランを放ち、チームの大量得点に貢献した。</t>
+          <t>8回を無失点に抑える快投で、相手打線を完璧に封じ込めた。</t>
         </is>
       </c>
     </row>
@@ -554,17 +554,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>牧 秀悟</t>
+          <t>上沢 直之</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DeNA</t>
+          <t>ソフトバンク</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>6回裏にダメ押しの3ランホームランを放ち、勝利を決定づける一打となった。</t>
+          <t>6回3失点8奪三振の力投で、試合を作り勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ソト</t>
+          <t>中村 奨成</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ロッテ</t>
+          <t>広島</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8回裏にダメ押しの2ランホームランを放ち、チームの勝利を決定づけた。</t>
+          <t>5打数4安打2打点と猛打賞を大きく超える活躍で、打線を牽引した。</t>
         </is>
       </c>
     </row>

</xml_diff>